<commit_message>
add DOI pub 19
</commit_message>
<xml_diff>
--- a/StatPub/SummaryPub.xlsx
+++ b/StatPub/SummaryPub.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11102"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jeremycarlot/Documents/Website/JayCrlt.github.io/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jeremycarlot/Documents/Website/JayCrlt.github.io/StatPub/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{76C65739-D2E9-9142-AED0-3F5CC2920085}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AFAFB54-C557-4743-AF85-C21067632A0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5180" yWindow="1800" windowWidth="28040" windowHeight="17440" xr2:uid="{AA7BDC4C-3198-3143-B6C5-3B280DE634B4}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
   <si>
     <t>pubid</t>
   </si>
@@ -170,6 +170,9 @@
   </si>
   <si>
     <t>10.26028/cybium/2017-413-003</t>
+  </si>
+  <si>
+    <t>10.1111/ele.70376</t>
   </si>
 </sst>
 </file>
@@ -521,7 +524,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E76F7CDC-2270-2A4C-873C-81EB6C9C0E5D}">
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="3.1640625" bestFit="1" customWidth="1"/>
@@ -794,18 +797,26 @@
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
-        <v>37</v>
-      </c>
-      <c r="C20" t="s">
-        <v>23</v>
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
+        <v>37</v>
+      </c>
+      <c r="C21" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
         <v>36</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C22" t="s">
         <v>22</v>
       </c>
     </row>

</xml_diff>